<commit_message>
fix(catering-checklists-en): ronda 1 de la revisión adversarial — 1 BLOQUEANTE + 11 MAYOR + 15 menor aplicados
Time as a public health control bien dicho (a las 4 h se tira; 6 h en frío vigilando 70 °F), reloj desde
que sale de temperatura, sobrantes del buffet se tiran, enfriamiento en dos fases, aviso al consumidor,
CF de cabeceras corregido (desviación declarada), orden del 08, guaranteed count único, rótulos del sales tax,
calendario US. Autotest 20/20; base, bar y cafetería idénticos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/catering-checklist-templates/01-catering-prep-production-checklist.xlsx
+++ b/astro-site/public/dl/catering-checklist-templates/01-catering-prep-production-checklist.xlsx
@@ -694,7 +694,7 @@
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>▸ Green cells are editable: assigned to, due by, notes.</t>
+          <t>▸ Green cells are editable: assigned to, time, notes.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Do the pre-cooking: confit, braises, sous-vide</t>
+          <t>Do the pre-cooking: confit, braises, sous-vide. Cool anything made ahead in shallow pans, an ice bath or the blast chiller: 135 °F to 70 °F within 2 h, then to 41 °F within 4 h more (FDA Food Code 3-501.14), and log it</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Pre-plate cold starters and canapes</t>
+          <t>Pre-plate cold appetizers and canapés</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
@@ -1999,7 +1999,7 @@
   </mergeCells>
   <conditionalFormatting sqref="A6:G51">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$E6="✓"</formula>
+      <formula>AND($E6="✓",$B6&lt;&gt;"Task")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>

<commit_message>
fix(checklists-en): §3-402.11 completo (3 opciones con la temperatura de cada tramo + registros 3-402.12) en base, cafetería y catering
6 celdas, 4 xlsx: restaurant-checklist-templates/02 (kit LIVE, errata de texto, sigue en 2.0),
coffee-shop/02, catering/01 y catering/06. Ajuste de texto forzado en 2 celdas que ya desbordaban en el ES.
Bar, pizza, burger y ghost idénticos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/catering-checklist-templates/01-catering-prep-production-checklist.xlsx
+++ b/astro-site/public/dl/catering-checklist-templates/01-catering-prep-production-checklist.xlsx
@@ -727,9 +727,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>▸ Fish served raw or undercooked (ceviche, tartare, marinated, cold-smoked) needs parasite destruction first: frozen at −4 °F or below for 7 days, or at −31 °F or below until solid plus 15 h (FDA Food Code 3-402.11). Ask the supplier for the freezing record, keep it 90 days and note the lot.</t>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>▸ Fish served raw or undercooked (ceviche, tartare, marinated, cold-smoked) needs parasite destruction first: frozen and stored at −4 °F or below for 7 days; or frozen at −31 °F or below until solid and stored at −31 °F or below for 15 h; or frozen at −31 °F or below until solid and stored at −4 °F or below for 24 h (FDA Food Code 3-402.11). Ask the supplier for the freezing record, keep it 90 days (FDA Food Code 3-402.12) and note the lot.</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Fish served raw or undercooked (ceviche, tartare, marinated, cold-smoked) — parasite destruction: get the supplier's freezing record (−4 °F or below for 7 days, or −31 °F or below until solid + 15 h; FDA Food Code 3-402.11) or freeze it yourself, keep the record 90 days and note the lot</t>
+          <t>Fish served raw or undercooked (ceviche, tartare, marinated, cold-smoked) — parasite destruction: get the supplier's freezing record (−4 °F or below for 7 days; or −31 °F or below until solid, then 15 h at −31 °F or below or 24 h at −4 °F or below; FDA Food Code 3-402.11) or freeze it yourself, keep the record 90 days (FDA Food Code 3-402.12) and note the lot</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">

</xml_diff>